<commit_message>
engine: blended pick values - auto-adjusts league vs industry weight by league age
Young leagues (1-3 seasons): 80% industry / 20% league data
Mid leagues (4-5 seasons): 60% industry / 40% league data
Mature leagues (6-8 seasons): 40% industry / 60% league data
Established leagues (9+): 20% industry / 80% league data

Industry baseline from KTC, theScore, FantasyCalc, DLF (March 2026).
Each pick now stores leagueRaw, industryVal, and blendWeights for transparency.
</commit_message>
<xml_diff>
--- a/reports/DHQ_Engine_Report.xlsx
+++ b/reports/DHQ_Engine_Report.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -50,6 +50,50 @@
       <name val="Arial"/>
       <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00D4AF37"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00D4AF37"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Courier New"/>
+      <b val="1"/>
+      <color rgb="001A1A1A"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Courier New"/>
+      <color rgb="00444444"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="002E86C1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00D4AF37"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00666666"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="16">
@@ -144,7 +188,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -166,11 +210,25 @@
         <color rgb="00DDDDDD"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -219,6 +277,32 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -96597,278 +96681,1060 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="B1:D93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="65" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="41" t="inlineStr">
-        <is>
-          <t>DHQ Engine Formula Breakdown</t>
+    <row r="1" ht="35" customHeight="1">
+      <c r="B1" s="44" t="inlineStr">
+        <is>
+          <t>DHQ ENGINE — FORMULA REFERENCE</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="42" t="inlineStr">
+      <c r="B3" s="45" t="inlineStr">
+        <is>
+          <t>OVERVIEW</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="46" t="inlineStr">
+        <is>
+          <t>The DHQ (Dynasty Headquarters) Engine calculates a value for every NFL player on a 0-10,000 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="46" t="inlineStr">
+        <is>
+          <t>Unlike generic rankings, DHQ values are calculated using YOUR leagues actual scoring settings,</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="46" t="inlineStr">
+        <is>
+          <t>draft history, roster construction, and positional scarcity. Every league gets different values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="46" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="B8" s="46" t="inlineStr">
+        <is>
+          <t>League: The Psycho League: Year VI | 16-team | Superflex | IDP | Half-PPR</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="46" t="inlineStr">
+        <is>
+          <t>Data Sources: 5 seasons of stats, 4 seasons of draft picks, 3 seasons of FAAB transactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="46" t="inlineStr">
+        <is>
+          <t>Total Players Scored: 1,977 | Draft Pick Slots Valued: 112 (7 rounds × 16 teams)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="45" t="inlineStr">
+        <is>
+          <t>MASTER FORMULA</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="B13" s="47" t="inlineStr">
+        <is>
+          <t>DHQ Value = Core Score + Scarcity + Peak Bonus + Consistency + Durability</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="48" t="inlineStr">
+        <is>
+          <t>Where Core Score = (wPPG × AgeFactor × SitMult) / TopComposite × 7500</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="45" t="inlineStr">
+        <is>
+          <t>COMPONENT BREAKDOWN</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="49" t="inlineStr">
         <is>
           <t>Component</t>
         </is>
       </c>
-      <c r="B3" s="42" t="inlineStr">
+      <c r="C17" s="49" t="inlineStr">
         <is>
           <t>Weight</t>
         </is>
       </c>
-      <c r="C3" s="42" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="43" t="inlineStr">
+      <c r="D17" s="49" t="inlineStr">
+        <is>
+          <t>How It Works</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="45" customHeight="1">
+      <c r="B18" s="50" t="inlineStr">
+        <is>
+          <t>CORE SCORE</t>
+        </is>
+      </c>
+      <c r="C18" s="51" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="D18" s="52" t="inlineStr">
+        <is>
+          <t>The primary value driver. Combines production (wPPG), age trajectory (AgeFactor), and league situation (SitMult). Normalized against the top player to a 0-7,500 scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="45" customHeight="1">
+      <c r="B20" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  wPPG (Weighted PPG)</t>
+        </is>
+      </c>
+      <c r="C20" s="54" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D20" s="55" t="inlineStr">
+        <is>
+          <t>Weighted average of PPG across last 5 seasons. Recent seasons weighted heavier than older ones. Best single season gets extra weight to protect elite ceilings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="45" customHeight="1">
+      <c r="B21" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AgeFactor</t>
+        </is>
+      </c>
+      <c r="C21" s="54" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D21" s="55" t="inlineStr">
+        <is>
+          <t>Multiplier based on age vs position-specific peak window. 1.0 during peak years. Decays at 6% per year after peak. Peak windows: QB=34, RB=27, WR=30, TE=30, IDP=30.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="45" customHeight="1">
+      <c r="B22" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SitMult (Situation)</t>
+        </is>
+      </c>
+      <c r="C22" s="54" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D22" s="55" t="inlineStr">
+        <is>
+          <t>League rank multiplier. Top 3 at position = 1.20×. Top 5 = 1.12×. Top 10 = 1.05×. Bottom 25% = 0.88×. Bottom 10% = 0.78×. Clamped between 0.40 and 1.60.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="45" customHeight="1">
+      <c r="B24" s="50" t="inlineStr">
+        <is>
+          <t>SCARCITY</t>
+        </is>
+      </c>
+      <c r="C24" s="51" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="D24" s="52" t="inlineStr">
+        <is>
+          <t>Positional premium on a 0-1,000 scale. In Superflex leagues, QB scarcity is tiered: Top 12 QBs = 750, QB13-24 = 400, QB25+ = 100. Other positions get a flat scarcity based on starter pool size. Unrostered players get 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="45" customHeight="1">
+      <c r="B26" s="50" t="inlineStr">
+        <is>
+          <t>PEAK BONUS</t>
+        </is>
+      </c>
+      <c r="C26" s="51" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="D26" s="52" t="inlineStr">
+        <is>
+          <t>120 DHQ per remaining peak year, capped at 1,000. A 23-year-old WR with 7 peak years left gets 840 bonus. A 31-year-old RB past peak gets 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="45" customHeight="1">
+      <c r="B28" s="50" t="inlineStr">
+        <is>
+          <t>CONSISTENCY</t>
+        </is>
+      </c>
+      <c r="C28" s="51" t="inlineStr">
+        <is>
+          <t>~4%</t>
+        </is>
+      </c>
+      <c r="D28" s="52" t="inlineStr">
+        <is>
+          <t>Rewards proven producers. 4+ starter seasons = 400. 3 seasons = 300. 2 seasons = 150. Only applies to rostered players — unrostered get 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="45" customHeight="1">
+      <c r="B30" s="50" t="inlineStr">
+        <is>
+          <t>DURABILITY</t>
+        </is>
+      </c>
+      <c r="C30" s="51" t="inlineStr">
+        <is>
+          <t>~1%</t>
+        </is>
+      </c>
+      <c r="D30" s="52" t="inlineStr">
+        <is>
+          <t>Small bonus for availability. 16+ games played in most recent season = 100. 13+ games = 50. Rewards iron men, penalizes injury-prone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="45" t="inlineStr">
+        <is>
+          <t>WORKED EXAMPLE: Josh Allen (DHQ 9,350)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="49" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="C33" s="49" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D33" s="49" t="inlineStr">
+        <is>
+          <t>Explanation</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="53" t="inlineStr">
+        <is>
+          <t>wPPG</t>
+        </is>
+      </c>
+      <c r="C34" s="53" t="inlineStr">
+        <is>
+          <t>25.6</t>
+        </is>
+      </c>
+      <c r="D34" s="53" t="inlineStr">
+        <is>
+          <t>Weighted PPG across 5 seasons — elite production</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="53" t="inlineStr">
+        <is>
+          <t>AgeFactor</t>
+        </is>
+      </c>
+      <c r="C35" s="53" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="D35" s="53" t="inlineStr">
+        <is>
+          <t>Age 29, QB peak window extends to 34 — still in prime</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="53" t="inlineStr">
+        <is>
+          <t>SitMult</t>
+        </is>
+      </c>
+      <c r="C36" s="53" t="inlineStr">
+        <is>
+          <t>1.558</t>
+        </is>
+      </c>
+      <c r="D36" s="53" t="inlineStr">
+        <is>
+          <t>Top 3 QB in this leagues scoring — elite situation bonus</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="53" t="inlineStr">
         <is>
           <t>Core Score</t>
         </is>
       </c>
-      <c r="B4" s="43" t="inlineStr">
-        <is>
-          <t>75%</t>
-        </is>
-      </c>
-      <c r="C4" s="43" t="inlineStr">
-        <is>
-          <t>wPPG × AgeFactor × SitMult, normalized to 0-7500 scale</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="43" t="inlineStr">
+      <c r="C37" s="53" t="inlineStr">
+        <is>
+          <t>~7,500</t>
+        </is>
+      </c>
+      <c r="D37" s="53" t="inlineStr">
+        <is>
+          <t>(25.6 × 1.0 × 1.558) / topComposite × 7500 = ~7,500</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="53" t="inlineStr">
+        <is>
+          <t>Scarcity</t>
+        </is>
+      </c>
+      <c r="C38" s="53" t="inlineStr">
+        <is>
+          <t>+750</t>
+        </is>
+      </c>
+      <c r="D38" s="53" t="inlineStr">
+        <is>
+          <t>Top 12 QB in Superflex — full QB scarcity premium</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="53" t="inlineStr">
+        <is>
+          <t>Peak Bonus</t>
+        </is>
+      </c>
+      <c r="C39" s="53" t="inlineStr">
+        <is>
+          <t>+600</t>
+        </is>
+      </c>
+      <c r="D39" s="53" t="inlineStr">
+        <is>
+          <t>5 peak years remaining × 120 = 600</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="53" t="inlineStr">
+        <is>
+          <t>Consistency</t>
+        </is>
+      </c>
+      <c r="C40" s="53" t="inlineStr">
+        <is>
+          <t>+400</t>
+        </is>
+      </c>
+      <c r="D40" s="53" t="inlineStr">
+        <is>
+          <t>4 starter seasons — maximum consistency bonus</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="53" t="inlineStr">
+        <is>
+          <t>Durability</t>
+        </is>
+      </c>
+      <c r="C41" s="53" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+      <c r="D41" s="53" t="inlineStr">
+        <is>
+          <t>17 games played — full durability bonus</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="56" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C42" s="56" t="inlineStr">
+        <is>
+          <t>9,350</t>
+        </is>
+      </c>
+      <c r="D42" s="56" t="inlineStr">
+        <is>
+          <t>7,500 + 750 + 600 + 400 + 100 = 9,350</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="45" t="inlineStr">
+        <is>
+          <t>POSITION PEAK WINDOWS &amp; AGE DECAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="49" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="C45" s="49" t="inlineStr">
+        <is>
+          <t>Peak Until</t>
+        </is>
+      </c>
+      <c r="D45" s="49" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="B46" s="57" t="inlineStr">
+        <is>
+          <t>QB</t>
+        </is>
+      </c>
+      <c r="C46" s="54" t="inlineStr">
+        <is>
+          <t>Age 34</t>
+        </is>
+      </c>
+      <c r="D46" s="55" t="inlineStr">
+        <is>
+          <t>Longest peak window. QBs hold value deep into their 30s. 6% annual decay after 34.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="B47" s="57" t="inlineStr">
+        <is>
+          <t>RB</t>
+        </is>
+      </c>
+      <c r="C47" s="54" t="inlineStr">
+        <is>
+          <t>Age 27</t>
+        </is>
+      </c>
+      <c r="D47" s="55" t="inlineStr">
+        <is>
+          <t>Shortest peak. RBs decline fastest. A 28-year-old RB is already decaying at 6%/year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="30" customHeight="1">
+      <c r="B48" s="57" t="inlineStr">
+        <is>
+          <t>WR</t>
+        </is>
+      </c>
+      <c r="C48" s="54" t="inlineStr">
+        <is>
+          <t>Age 30</t>
+        </is>
+      </c>
+      <c r="D48" s="55" t="inlineStr">
+        <is>
+          <t>Middle ground. WRs can produce into early 30s but decline accelerates after 30.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="B49" s="57" t="inlineStr">
+        <is>
+          <t>TE</t>
+        </is>
+      </c>
+      <c r="C49" s="54" t="inlineStr">
+        <is>
+          <t>Age 30</t>
+        </is>
+      </c>
+      <c r="D49" s="55" t="inlineStr">
+        <is>
+          <t>Similar to WR. Late bloomers common at TE so the engine accounts for this.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="B50" s="57" t="inlineStr">
+        <is>
+          <t>DL/LB/DB</t>
+        </is>
+      </c>
+      <c r="C50" s="54" t="inlineStr">
+        <is>
+          <t>Age 30</t>
+        </is>
+      </c>
+      <c r="D50" s="55" t="inlineStr">
+        <is>
+          <t>IDP players follow a similar curve to offensive skill positions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="B51" s="57" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="C51" s="54" t="inlineStr">
+        <is>
+          <t>Age 30</t>
+        </is>
+      </c>
+      <c r="D51" s="55" t="inlineStr">
+        <is>
+          <t>Kickers have long careers but limited dynasty value regardless of age.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="45" t="inlineStr">
+        <is>
+          <t>DRAFT PICK VALUATION METHODOLOGY</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="46" t="inlineStr">
+        <is>
+          <t>Draft pick values are NOT static numbers — they are calculated from YOUR leagues actual draft history.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="58" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="B56" s="46" t="inlineStr">
+        <is>
+          <t>For each draft slot (1-112), the engine looks at every player drafted at that slot across 4 seasons and asks:</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1. HIT RATE — What % of picks at this slot became top-15% players at their position?</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2. STARTER RATE — What % became starter-level producers (above the starter line)?</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  3. AVG NORMALIZED PPG — Average production relative to the position starter threshold.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="58" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="B61" s="46" t="inlineStr">
+        <is>
+          <t>These three metrics are combined into a single DHQ value for each pick slot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="58" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="B63" s="46" t="inlineStr">
+        <is>
+          <t>Key insight: An early 1st (slot 1-4) is worth 9,000-9,975 DHQ in your league.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="46" t="inlineStr">
+        <is>
+          <t>A late 1st (slot 13-16) is worth 5,688-6,600 — a massive difference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="46" t="inlineStr">
+        <is>
+          <t>This is why "a 1st round pick" is not a single value — position within the round matters.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="58" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="B67" s="46" t="inlineStr">
+        <is>
+          <t>War Room uses flat values (1st = 5,500 for all). DHQ uses slot-specific values derived from your leagues history.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="46" t="inlineStr">
+        <is>
+          <t>This means ReconAI and War Room will value the same pick differently until the engines are unified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="45" t="inlineStr">
+        <is>
+          <t>VALUE SCALE REFERENCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="25" customHeight="1">
+      <c r="B71" s="49" t="inlineStr">
+        <is>
+          <t>DHQ Range</t>
+        </is>
+      </c>
+      <c r="C71" s="49" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="D71" s="49" t="inlineStr">
+        <is>
+          <t>Examples</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="25" customHeight="1">
+      <c r="B72" s="59" t="inlineStr">
+        <is>
+          <t>8,000 - 10,000</t>
+        </is>
+      </c>
+      <c r="C72" s="55" t="inlineStr">
+        <is>
+          <t>ELITE — Franchise cornerstone</t>
+        </is>
+      </c>
+      <c r="D72" s="55" t="inlineStr">
+        <is>
+          <t>Josh Allen (9,350), Bijan Robinson (7,673)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="25" customHeight="1">
+      <c r="B73" s="59" t="inlineStr">
+        <is>
+          <t>6,000 - 8,000</t>
+        </is>
+      </c>
+      <c r="C73" s="55" t="inlineStr">
+        <is>
+          <t>STAR — Top 20 dynasty asset</t>
+        </is>
+      </c>
+      <c r="D73" s="55" t="inlineStr">
+        <is>
+          <t>Ja'Marr Chase (7,065), Trevor Lawrence (6,528)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="25" customHeight="1">
+      <c r="B74" s="59" t="inlineStr">
+        <is>
+          <t>4,000 - 6,000</t>
+        </is>
+      </c>
+      <c r="C74" s="55" t="inlineStr">
+        <is>
+          <t>STARTER — Reliable weekly starter</t>
+        </is>
+      </c>
+      <c r="D74" s="55" t="inlineStr">
+        <is>
+          <t>CeeDee Lamb range, emerging young players</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="25" customHeight="1">
+      <c r="B75" s="59" t="inlineStr">
+        <is>
+          <t>2,000 - 4,000</t>
+        </is>
+      </c>
+      <c r="C75" s="55" t="inlineStr">
+        <is>
+          <t>DEPTH — Flex play / upside stash</t>
+        </is>
+      </c>
+      <c r="D75" s="55" t="inlineStr">
+        <is>
+          <t>Veteran starters, young backups with upside</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="25" customHeight="1">
+      <c r="B76" s="59" t="inlineStr">
+        <is>
+          <t>500 - 2,000</t>
+        </is>
+      </c>
+      <c r="C76" s="55" t="inlineStr">
+        <is>
+          <t>ROSTER FILLER — Bench depth</t>
+        </is>
+      </c>
+      <c r="D76" s="55" t="inlineStr">
+        <is>
+          <t>Backup QBs, aging veterans, IDP starters</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="25" customHeight="1">
+      <c r="B77" s="59" t="inlineStr">
+        <is>
+          <t>0 - 500</t>
+        </is>
+      </c>
+      <c r="C77" s="55" t="inlineStr">
+        <is>
+          <t>WAIVER LEVEL — Minimal value</t>
+        </is>
+      </c>
+      <c r="D77" s="55" t="inlineStr">
+        <is>
+          <t>Practice squad, late-round IDP, kickers</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" s="45" t="inlineStr">
+        <is>
+          <t>COLUMN DEFINITIONS (All Players Sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="22" customHeight="1">
+      <c r="B80" s="49" t="inlineStr">
+        <is>
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="C80" s="49" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D80" s="49" t="inlineStr">
+        <is>
+          <t>Definition</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="22" customHeight="1">
+      <c r="B81" s="59" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="C81" s="55" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="D81" s="55" t="inlineStr">
+        <is>
+          <t>Overall DHQ rank among all 1,977 scored players</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="22" customHeight="1">
+      <c r="B82" s="59" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="C82" s="55" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D82" s="55" t="inlineStr">
+        <is>
+          <t>Player full name</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="22" customHeight="1">
+      <c r="B83" s="59" t="inlineStr">
+        <is>
+          <t>Pos</t>
+        </is>
+      </c>
+      <c r="C83" s="55" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D83" s="55" t="inlineStr">
+        <is>
+          <t>Position: QB, RB, WR, TE, DL, LB, DB, K</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="22" customHeight="1">
+      <c r="B84" s="59" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="C84" s="55" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D84" s="55" t="inlineStr">
+        <is>
+          <t>Current NFL team (FA = free agent)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="22" customHeight="1">
+      <c r="B85" s="59" t="inlineStr">
+        <is>
+          <t>Age</t>
+        </is>
+      </c>
+      <c r="C85" s="55" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="D85" s="55" t="inlineStr">
+        <is>
+          <t>Current age</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="22" customHeight="1">
+      <c r="B86" s="59" t="inlineStr">
+        <is>
+          <t>DHQ Value</t>
+        </is>
+      </c>
+      <c r="C86" s="55" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="D86" s="55" t="inlineStr">
+        <is>
+          <t>Final dynasty value on 0-10,000 scale</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="22" customHeight="1">
+      <c r="B87" s="59" t="inlineStr">
         <is>
           <t>wPPG</t>
         </is>
       </c>
-      <c r="B5" s="43" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C5" s="43" t="inlineStr">
-        <is>
-          <t>Weighted avg PPG across 5 seasons. Recent years weighted more. Best season gets bonus weight.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="43" t="inlineStr">
+      <c r="C87" s="55" t="inlineStr">
+        <is>
+          <t>Decimal</t>
+        </is>
+      </c>
+      <c r="D87" s="55" t="inlineStr">
+        <is>
+          <t>Weighted points per game — production input to the formula</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="22" customHeight="1">
+      <c r="B88" s="59" t="inlineStr">
         <is>
           <t>AgeFactor</t>
         </is>
       </c>
-      <c r="B6" s="43" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C6" s="43" t="inlineStr">
-        <is>
-          <t>1.0 during peak years. Decays after position peak: QB=34, RB=27, WR=30, TE=30. Rate: 6%/year.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="43" t="inlineStr">
+      <c r="C88" s="55" t="inlineStr">
+        <is>
+          <t>Decimal</t>
+        </is>
+      </c>
+      <c r="D88" s="55" t="inlineStr">
+        <is>
+          <t>1.0 = in peak. &lt;1.0 = declining. Decays 6%/year after peak age.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="22" customHeight="1">
+      <c r="B89" s="59" t="inlineStr">
         <is>
           <t>SitMult</t>
         </is>
       </c>
-      <c r="B7" s="43" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C7" s="43" t="inlineStr">
-        <is>
-          <t>Positional rank multiplier: Top3=1.20x, Top5=1.12x, Top10=1.05x, Bottom25%=0.88x. Clamped 0.40-1.60.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="43" t="inlineStr">
-        <is>
-          <t>Scarcity</t>
-        </is>
-      </c>
-      <c r="B8" s="43" t="inlineStr">
-        <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="C8" s="43" t="inlineStr">
-        <is>
-          <t>Position premium (0-1000). QB tiered in SF: Top12=750, QB13-24=400, QB25+=100. Zero for unrostered.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="43" t="inlineStr">
-        <is>
-          <t>Peak Bonus</t>
-        </is>
-      </c>
-      <c r="B9" s="43" t="inlineStr">
-        <is>
-          <t>5%</t>
-        </is>
-      </c>
-      <c r="C9" s="43" t="inlineStr">
-        <is>
-          <t>120 DHQ per peak year remaining, capped at 1000.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="43" t="inlineStr">
-        <is>
-          <t>Consistency</t>
-        </is>
-      </c>
-      <c r="B10" s="43" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C10" s="43" t="inlineStr">
-        <is>
-          <t>4+ starter seasons = 400, 3 = 300, 2 = 150. Zero for unrostered players.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="43" t="inlineStr">
-        <is>
-          <t>Durability</t>
-        </is>
-      </c>
-      <c r="B11" s="43" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C11" s="43" t="inlineStr">
-        <is>
-          <t>16+ recent GP = 100, 13+ = 50.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="43" t="inlineStr"/>
-      <c r="B12" s="43" t="inlineStr"/>
-      <c r="C12" s="43" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="43" t="inlineStr">
-        <is>
-          <t>PICK VALUES</t>
-        </is>
-      </c>
-      <c r="B13" s="43" t="inlineStr"/>
-      <c r="C13" s="43" t="inlineStr">
-        <is>
-          <t>Based on YOUR leagues actual 4-season draft history</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="43" t="inlineStr">
-        <is>
-          <t>Hit Rate</t>
-        </is>
-      </c>
-      <c r="B14" s="43" t="inlineStr"/>
-      <c r="C14" s="43" t="inlineStr">
-        <is>
-          <t>% of picks at that slot that produced a top-15% player at their position</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="43" t="inlineStr">
-        <is>
-          <t>Starter Rate</t>
-        </is>
-      </c>
-      <c r="B15" s="43" t="inlineStr"/>
-      <c r="C15" s="43" t="inlineStr">
-        <is>
-          <t>% of picks at that slot that produced a starter-level season</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="43" t="inlineStr">
-        <is>
-          <t>AvgNormPPG</t>
-        </is>
-      </c>
-      <c r="B16" s="43" t="inlineStr"/>
-      <c r="C16" s="43" t="inlineStr">
-        <is>
-          <t>Average normalized PPG produced by picks at that draft slot</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="43" t="inlineStr"/>
-      <c r="B17" s="43" t="inlineStr"/>
-      <c r="C17" s="43" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="43" t="inlineStr">
-        <is>
-          <t>SCALE</t>
-        </is>
-      </c>
-      <c r="B18" s="43" t="inlineStr"/>
-      <c r="C18" s="43" t="inlineStr">
-        <is>
-          <t>All DHQ values are 0-10,000. Top player ~9,500. Average starter ~3,000-4,000.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="43" t="inlineStr">
-        <is>
-          <t>LEAGUE</t>
-        </is>
-      </c>
-      <c r="B19" s="43" t="inlineStr"/>
-      <c r="C19" s="43" t="inlineStr">
-        <is>
-          <t>The Psycho League: Year VI — 16-team Superflex IDP Half-PPR</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="43" t="inlineStr">
-        <is>
-          <t>ENGINE</t>
-        </is>
-      </c>
-      <c r="B20" s="43" t="inlineStr"/>
-      <c r="C20" s="43" t="inlineStr">
-        <is>
-          <t>Values recalculated using YOUR league scoring settings, not generic rankings</t>
+      <c r="C89" s="55" t="inlineStr">
+        <is>
+          <t>Decimal</t>
+        </is>
+      </c>
+      <c r="D89" s="55" t="inlineStr">
+        <is>
+          <t>Situation multiplier. &gt;1.0 = elite rank. &lt;1.0 = below average rank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="22" customHeight="1">
+      <c r="B90" s="59" t="inlineStr">
+        <is>
+          <t>Peak Yrs Left</t>
+        </is>
+      </c>
+      <c r="C90" s="55" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="D90" s="55" t="inlineStr">
+        <is>
+          <t>Years remaining in position-specific peak window</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="22" customHeight="1">
+      <c r="B91" s="59" t="inlineStr">
+        <is>
+          <t>Starter Seasons</t>
+        </is>
+      </c>
+      <c r="C91" s="55" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="D91" s="55" t="inlineStr">
+        <is>
+          <t>Number of seasons player produced starter-level output</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="22" customHeight="1">
+      <c r="B92" s="59" t="inlineStr">
+        <is>
+          <t>Recent GP</t>
+        </is>
+      </c>
+      <c r="C92" s="55" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="D92" s="55" t="inlineStr">
+        <is>
+          <t>Games played in most recent season (durability indicator)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="22" customHeight="1">
+      <c r="B93" s="59" t="inlineStr">
+        <is>
+          <t>Trend %</t>
+        </is>
+      </c>
+      <c r="C93" s="55" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="D93" s="55" t="inlineStr">
+        <is>
+          <t>Year-over-year PPG change. +15 = 15% improvement. -20 = 20% decline.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+  <mergeCells count="33">
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B60:D60"/>
+    <mergeCell ref="B67:D67"/>
+    <mergeCell ref="B61:D61"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B57:D57"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="B53:D53"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B65:D65"/>
+    <mergeCell ref="B68:D68"/>
+    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B64:D64"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B63:D63"/>
+    <mergeCell ref="B79:D79"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B62:D62"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B54:D54"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B59:D59"/>
+    <mergeCell ref="B66:D66"/>
+    <mergeCell ref="B56:D56"/>
+    <mergeCell ref="B58:D58"/>
+    <mergeCell ref="B70:D70"/>
+    <mergeCell ref="B12:D12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>